<commit_message>
fix: generate sample data at second precision
Minute-rounded HH:MM storage collapsed the continuous exponential sample to
ties, so chi-square rejected the fitted exponential at p ≈ 0 for both
inter-arrival and service times — a correct test against genuinely discrete
empirical data. Switch the generator to HH:MM:SS (1/60 min quantisation,
D-048); the RNG stream is untouched, so the underlying seed-42 draws are
identical. TimeParser already understood H:mm:ss; a TimeParserTests case
(8:17:30 → 497.5) now pins it without disturbing the HH:MM cases. Samples
and the dirty fixture were regenerated. 98 tests green, 0 warnings.
</commit_message>
<xml_diff>
--- a/samples/sample_patients.xlsx
+++ b/samples/sample_patients.xlsx
@@ -28,250 +28,541 @@
     <x:t>screening_end</x:t>
   </x:si>
   <x:si>
-    <x:t>8:17</x:t>
+    <x:t>8:17:12</x:t>
   </x:si>
   <x:si>
     <x:t>Screening</x:t>
   </x:si>
   <x:si>
-    <x:t>8:18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:19</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:23</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:24</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:25</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:26</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:27</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:29</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:31</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:33</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:34</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:35</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:40</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:41</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:38</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:43</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:44</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:46</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:48</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:45</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:50</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:49</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:52</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:51</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:53</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:54</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:56</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:58</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:55</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:57</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8:59</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:07</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:08</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:09</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:13</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:25</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:16</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:17</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:19</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:23</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:28</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:31</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:33</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:40</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:41</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:42</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:45</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:43</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:50</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:44</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:46</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:48</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:53</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:54</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:49</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:58</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:04</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:55</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:59</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9:57</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:06</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:05</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:09</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:02</x:t>
+    <x:t>8:17:58</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:18:12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:18:41</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:19:48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:20:04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:21:16</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:22:09</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:23:13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:24:08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:25:13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:25:37</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:25:32</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:27:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:27:34</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:26:08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:26:43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:27:48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:29:30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:31:01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:32:19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:29:50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:32:47</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:32:55</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:33:13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:33:49</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:34:59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:35:42</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:40:56</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:41:11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:38:04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:38:59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:40:04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:38:09</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:40:24</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:40:57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:41:36</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:43:38</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:44:52</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:46:20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:48:24</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:45:11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:45:47</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:45:50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:48:14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:48:58</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:50:27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:48:48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:49:59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:52:13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:50:54</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:51:29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:51:43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:52:45</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:53:21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:54:27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:53:50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:56:19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:58:10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:54:20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:55:45</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:55:46</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:54:57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:57:59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:58:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:55:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:55:38</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:56:34</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:58:18</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:00:14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:01:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:59:41</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:03:43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:03:44</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8:59:43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:00:21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:01:50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:07:14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:07:17</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:07:07</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:08:34</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:09:30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:09:02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:10:28</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:10:32</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:09:21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:12:59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:13:51</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:10:52</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:12:04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:12:50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:15:37</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:18:47</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:20:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:15:40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:22:29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:25:41</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:16:28</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:17:20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:19:11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:16:41</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:18:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:18:54</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:19:41</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:20:28</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:20:43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:20:10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:22:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:23:27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:28:51</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:31:35</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:33:46</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:31:22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:33:28</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:33:59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:40:33</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:41:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:42:40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:41:23</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:41:57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:45:55</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:41:53</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:42:28</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:42:56</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:42:22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:43:58</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:45:19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:42:34</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:43:20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:50:53</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:42:48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:44:05</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:44:40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:45:35</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:46:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:48:43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:45:40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:50:41</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:53:26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:46:12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:50:26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:54:21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:46:52</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:49:23</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:50:33</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:48:50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:50:02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:50:21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:49:14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:50:15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:50:18</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:54:39</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:58:12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:04:45</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:54:56</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:55:51</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:59:05</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:55:38</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:57:46</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:59:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:58:08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:00:27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:00:39</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:59:08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:00:48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:04:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9:59:59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:01:44</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:06:42</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:01:33</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:05:22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:09:48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:01:49</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:02:20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:02:30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:02:13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:05:16</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:09:30</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -647,836 +938,836 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4">
       <x:c r="A3" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:4">
       <x:c r="A4" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:4">
       <x:c r="A5" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:4">
       <x:c r="A6" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:4">
       <x:c r="A7" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:4">
       <x:c r="A8" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:4">
       <x:c r="A9" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:4">
       <x:c r="A10" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:4">
       <x:c r="A11" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:4">
       <x:c r="A12" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:4">
       <x:c r="A13" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:4">
       <x:c r="A14" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:4">
       <x:c r="A15" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:4">
       <x:c r="A16" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:4">
       <x:c r="A17" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:4">
       <x:c r="A18" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:4">
       <x:c r="A19" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:4">
       <x:c r="A20" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:4">
       <x:c r="A21" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C21" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:4">
       <x:c r="A22" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C22" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:4">
       <x:c r="A23" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C23" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:4">
       <x:c r="A24" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C24" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:4">
       <x:c r="A25" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C25" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:4">
       <x:c r="A26" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:4">
       <x:c r="A27" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C27" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:4">
       <x:c r="A28" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B28" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C28" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:4">
       <x:c r="A29" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B29" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C29" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:4">
       <x:c r="A30" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C30" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:4">
       <x:c r="A31" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C31" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:4">
       <x:c r="A32" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C32" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:4">
       <x:c r="A33" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B33" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C33" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:4">
       <x:c r="A34" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C34" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:4">
       <x:c r="A35" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C35" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:4">
       <x:c r="A36" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C36" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:4">
       <x:c r="A37" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B37" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C37" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:4">
       <x:c r="A38" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C38" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:4">
       <x:c r="A39" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B39" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C39" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:4">
       <x:c r="A40" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C40" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="D40" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>119</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:4">
       <x:c r="A41" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B41" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C41" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D41" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>122</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:4">
       <x:c r="A42" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="B42" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C42" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="D42" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>125</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:4">
       <x:c r="A43" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="B43" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C43" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="D43" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:4">
       <x:c r="A44" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B44" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C44" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D44" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>131</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:4">
       <x:c r="A45" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B45" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C45" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D45" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:4">
       <x:c r="A46" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B46" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C46" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D46" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:4">
       <x:c r="A47" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B47" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C47" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="D47" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>140</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:4">
       <x:c r="A48" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B48" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C48" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="D48" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:4">
       <x:c r="A49" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="B49" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C49" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="D49" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:4">
       <x:c r="A50" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B50" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C50" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D50" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:4">
       <x:c r="A51" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B51" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C51" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="D51" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>152</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:4">
       <x:c r="A52" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B52" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C52" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="D52" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>155</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:4">
       <x:c r="A53" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B53" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C53" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="D53" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:4">
       <x:c r="A54" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B54" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C54" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D54" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:4">
       <x:c r="A55" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B55" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C55" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="D55" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:4">
       <x:c r="A56" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B56" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C56" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="D56" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:4">
       <x:c r="A57" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B57" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C57" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="D57" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>170</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:4">
       <x:c r="A58" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B58" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C58" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="D58" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:4">
       <x:c r="A59" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B59" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C59" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="D59" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:4">
       <x:c r="A60" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B60" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C60" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="D60" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>179</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:4">
       <x:c r="A61" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="B61" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C61" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D61" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>